<commit_message>
update format of excel file
</commit_message>
<xml_diff>
--- a/st-interp/2025_data_interpolation_comparison.xlsx
+++ b/st-interp/2025_data_interpolation_comparison.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smt3/Documents/GitHub/atomic-clock/st-interp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{614D3C29-0945-3041-85ED-1F489365D309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B1F0BA-E4F5-B449-B00C-7C451EDDE49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6520" yWindow="-19360" windowWidth="28040" windowHeight="16940" activeTab="1" xr2:uid="{A8975FA8-588C-2342-9420-A35ABBC5CCC5}"/>
   </bookViews>
@@ -121,7 +121,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -138,11 +138,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -151,9 +171,11 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2406,6 +2428,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="12" max="12" width="17.5" customWidth="1"/>
+    <col min="13" max="13" width="6.6640625" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.2">
@@ -2745,7 +2769,7 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
+      <c r="M7" s="8"/>
       <c r="N7" s="5">
         <f t="shared" si="0"/>
         <v>0.58323000000000003</v>
@@ -3051,7 +3075,7 @@
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
       <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+      <c r="M13" s="8"/>
       <c r="N13" s="5">
         <f t="shared" si="0"/>
         <v>0.42806</v>
@@ -3357,7 +3381,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
+      <c r="M19" s="8"/>
       <c r="N19" s="5">
         <f t="shared" si="0"/>
         <v>0.18430999999999997</v>
@@ -3663,7 +3687,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="M25" s="8"/>
       <c r="N25" s="5">
         <f t="shared" si="0"/>
         <v>0.23746</v>
@@ -3969,7 +3993,7 @@
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
+      <c r="M31" s="8"/>
       <c r="N31" s="5">
         <f t="shared" si="0"/>
         <v>0.76456000000000002</v>
@@ -4275,7 +4299,7 @@
       <c r="J37" s="2"/>
       <c r="K37" s="2"/>
       <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
+      <c r="M37" s="8"/>
       <c r="N37" s="5">
         <f t="shared" si="6"/>
         <v>1.1113999999999999</v>
@@ -4581,7 +4605,7 @@
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
+      <c r="M43" s="8"/>
       <c r="N43" s="5">
         <f t="shared" si="6"/>
         <v>0.14147000000000001</v>
@@ -4887,7 +4911,7 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
-      <c r="M49" s="2"/>
+      <c r="M49" s="8"/>
       <c r="N49" s="5">
         <f t="shared" si="6"/>
         <v>0.35600000000000004</v>
@@ -5193,7 +5217,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
+      <c r="M55" s="8"/>
       <c r="N55" s="5">
         <f t="shared" si="6"/>
         <v>0.68614000000000008</v>
@@ -5499,7 +5523,7 @@
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
       <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
+      <c r="M61" s="8"/>
       <c r="N61" s="5">
         <f t="shared" si="6"/>
         <v>0.48627000000000004</v>
@@ -5805,7 +5829,7 @@
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
       <c r="L67" s="2"/>
-      <c r="M67" s="2"/>
+      <c r="M67" s="8"/>
       <c r="N67" s="5">
         <f t="shared" si="6"/>
         <v>0.75347999999999993</v>

</xml_diff>